<commit_message>
Allow skipping of scoring for particular choice and scale pair (#4768)
* Allow skipping of scoring for particular choice and scale pair

* Code review changes
</commit_message>
<xml_diff>
--- a/spec/fixtures/files/import_assessment_questions/valid_file.xlsx
+++ b/spec/fixtures/files/import_assessment_questions/valid_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohanpujari/tte/psychometrics/spec/fixtures/files/import_assessment_questions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohan-pujari/tte/psychometrics/spec/fixtures/files/import_assessment_questions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D154129C-2018-2A47-A428-E054813A4135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5CE01CF-F5C7-B14A-8628-D766FE1C6E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="35120" windowHeight="22500" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="33620" windowHeight="21580" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -218,12 +218,6 @@
     <t>All</t>
   </si>
   <si>
-    <t>3,2,4,6,3,5</t>
-  </si>
-  <si>
-    <t>1,2, 3</t>
-  </si>
-  <si>
     <t>2, 4,5</t>
   </si>
   <si>
@@ -258,6 +252,12 @@
   </si>
   <si>
     <t>Strongly Agree</t>
+  </si>
+  <si>
+    <t>1,, 3</t>
+  </si>
+  <si>
+    <t>,,,4,,5</t>
   </si>
 </sst>
 </file>
@@ -804,7 +804,7 @@
         <v>27</v>
       </c>
       <c r="O4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -858,10 +858,10 @@
         <v>45</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="Q6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -890,7 +890,7 @@
         <v>57</v>
       </c>
       <c r="M7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -924,7 +924,7 @@
         <v>59</v>
       </c>
       <c r="O8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
@@ -932,7 +932,7 @@
         <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D9" s="1"/>
       <c r="G9" s="1"/>
@@ -959,10 +959,10 @@
         <v>40</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
@@ -981,7 +981,7 @@
         <v>33</v>
       </c>
       <c r="Q10" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -1004,22 +1004,22 @@
         <v>41</v>
       </c>
       <c r="G11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L11" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -1027,7 +1027,7 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>48</v>
@@ -1036,7 +1036,7 @@
         <v>43</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>

</xml_diff>

<commit_message>
Allow period in factor score (#4846)
* Allow period in factor score

* Fix specs

* Don't escape for scoring
</commit_message>
<xml_diff>
--- a/spec/fixtures/files/import_assessment_questions/valid_file.xlsx
+++ b/spec/fixtures/files/import_assessment_questions/valid_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohan-pujari/tte/psychometrics/spec/fixtures/files/import_assessment_questions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5CE01CF-F5C7-B14A-8628-D766FE1C6E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DA584B6-3515-C94C-9095-86FD2E11D4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="33620" windowHeight="21580" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="52700" windowHeight="24580" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -98,9 +98,6 @@
     <t>answersType</t>
   </si>
   <si>
-    <t>Grit</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -258,6 +255,9 @@
   </si>
   <si>
     <t>,,,4,,5</t>
+  </si>
+  <si>
+    <t>.Grit.1</t>
   </si>
 </sst>
 </file>
@@ -705,7 +705,7 @@
         <v>12</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P1" t="s">
         <v>13</v>
@@ -743,28 +743,28 @@
         <v>14</v>
       </c>
       <c r="J2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M2" t="s">
         <v>15</v>
       </c>
       <c r="N2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="O2" t="s">
         <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q2" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -775,16 +775,16 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -792,19 +792,19 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -812,16 +812,16 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
@@ -829,39 +829,39 @@
         <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="O6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Q6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -869,28 +869,28 @@
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="I7" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N7">
         <v>1</v>
@@ -902,29 +902,29 @@
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="I8" s="1"/>
       <c r="M8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="O8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
@@ -932,7 +932,7 @@
         <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D9" s="1"/>
       <c r="G9" s="1"/>
@@ -944,25 +944,25 @@
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
@@ -975,13 +975,13 @@
         <v>6</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="P10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="Q10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -989,37 +989,37 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="I11" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I11" s="1" t="s">
+      <c r="J11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="L11" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="J11" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -1027,16 +1027,16 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>

</xml_diff>

<commit_message>
Add not applicable option to question import (#5014)
* Add not applicable option to question import

* Cache allowed factors
</commit_message>
<xml_diff>
--- a/spec/fixtures/files/import_assessment_questions/valid_file.xlsx
+++ b/spec/fixtures/files/import_assessment_questions/valid_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohan-pujari/tte/psychometrics/spec/fixtures/files/import_assessment_questions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F738365-DC0B-D74B-A8EF-E00835009AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E572BF0-4991-F341-9FCB-3738A3D381E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="52700" windowHeight="24580" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="33620" windowHeight="21580" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="75">
   <si>
     <t>Q1</t>
   </si>
@@ -251,6 +251,18 @@
   </si>
   <si>
     <t>Factors</t>
+  </si>
+  <si>
+    <t>notApplicable</t>
+  </si>
+  <si>
+    <t>notApplicableLabel</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Q10</t>
   </si>
 </sst>
 </file>
@@ -642,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2760F84-0E72-1247-B859-B08C7CC9D341}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -654,13 +666,13 @@
     <col min="8" max="9" width="27.33203125" customWidth="1"/>
     <col min="10" max="10" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" customWidth="1"/>
-    <col min="13" max="15" width="37" customWidth="1"/>
-    <col min="16" max="16" width="24" customWidth="1"/>
-    <col min="17" max="17" width="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="25.83203125" customWidth="1"/>
+    <col min="15" max="17" width="37" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="19" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -704,13 +716,19 @@
         <v>12</v>
       </c>
       <c r="O1" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" t="s">
         <v>44</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -748,19 +766,25 @@
         <v>55</v>
       </c>
       <c r="M2" t="s">
+        <v>71</v>
+      </c>
+      <c r="N2" t="s">
+        <v>72</v>
+      </c>
+      <c r="O2" t="s">
         <v>15</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" t="s">
         <v>42</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
         <v>1</v>
       </c>
-      <c r="P2" t="s">
+      <c r="R2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -776,11 +800,11 @@
       <c r="E3" t="s">
         <v>25</v>
       </c>
-      <c r="O3" t="s">
+      <c r="Q3" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -796,11 +820,11 @@
       <c r="E4" t="s">
         <v>26</v>
       </c>
-      <c r="O4" t="s">
+      <c r="Q4" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -817,7 +841,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -844,17 +868,23 @@
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
-      <c r="M6" t="s">
+      <c r="M6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O6" t="s">
         <v>40</v>
       </c>
-      <c r="O6" t="s">
+      <c r="Q6" t="s">
         <v>43</v>
       </c>
-      <c r="P6" s="2" t="s">
+      <c r="R6" s="2" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -879,15 +909,18 @@
       <c r="I7" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="M7" t="s">
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="s">
         <v>59</v>
       </c>
-      <c r="N7">
+      <c r="P7">
         <v>1</v>
       </c>
-      <c r="P7" s="1"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="R7" s="1"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -910,14 +943,14 @@
         <v>30</v>
       </c>
       <c r="I8" s="1"/>
-      <c r="M8" t="s">
+      <c r="O8" t="s">
         <v>56</v>
       </c>
-      <c r="O8" t="s">
+      <c r="Q8" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -929,7 +962,7 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -964,14 +997,20 @@
       <c r="L10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="O10" s="1" t="s">
+      <c r="M10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="Q10" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="P10" s="3" t="s">
+      <c r="R10" s="3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1008,8 +1047,12 @@
       <c r="L11" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="M11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" s="1"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -1031,6 +1074,48 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>